<commit_message>
Remove binary demo outputs and update stratetab Excel file
</commit_message>
<xml_diff>
--- a/tabtools/demo/stratetab.xlsx
+++ b/tabtools/demo/stratetab.xlsx
@@ -100,953 +100,1007 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="225">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <b/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <b/>
+  <fonts count="238">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <b/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1074,7 +1128,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="162">
+  <borders count="175">
     <border>
       <left/>
       <right/>
@@ -2155,11 +2209,102 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -2775,6 +2920,58 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="224" fillId="0" borderId="161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="225" fillId="0" borderId="162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="226" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="227" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="228" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="229" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="230" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="231" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="232" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="233" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="234" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="235" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="236" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="237" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2848,7 +3045,7 @@
       <c r="G2" s="107" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="108" t="s">
+      <c r="H2" s="162" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2874,7 +3071,7 @@
       <c r="G3" s="114" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="115" t="s">
+      <c r="H3" s="163" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2900,7 +3097,7 @@
       <c r="G4" s="121" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="122" t="s">
+      <c r="H4" s="164" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2926,7 +3123,7 @@
       <c r="G5" s="128" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="129" t="s">
+      <c r="H5" s="165" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2952,7 +3149,7 @@
       <c r="G6" s="135" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="136" t="s">
+      <c r="H6" s="166" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2960,25 +3157,25 @@
       <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="155" t="s">
+      <c r="B7" s="168" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="138" t="s">
+      <c r="C7" s="169" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="139" t="s">
+      <c r="D7" s="170" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="161" t="s">
+      <c r="E7" s="171" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="141" t="s">
+      <c r="F7" s="172" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="142" t="s">
+      <c r="G7" s="173" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="143" t="s">
+      <c r="H7" s="174" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>